<commit_message>
sensitivity tests; full knit of record
</commit_message>
<xml_diff>
--- a/tables/Table S8.xlsx
+++ b/tables/Table S8.xlsx
@@ -60,7 +60,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -117,11 +117,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -151,6 +164,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -548,7 +568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col width="9" bestFit="1" customWidth="1" style="8" min="1" max="1"/>
@@ -622,197 +642,354 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>Habitat</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="15" t="inlineStr">
         <is>
           <t>Urban vs Reef</t>
         </is>
       </c>
-      <c r="C3" s="7" t="n">
-        <v>135</v>
-      </c>
-      <c r="D3" s="7" t="n">
-        <v>265</v>
-      </c>
-      <c r="E3" s="7" t="n">
-        <v>400</v>
-      </c>
-      <c r="F3" s="7" t="n">
-        <v>79</v>
-      </c>
-      <c r="G3" s="7" t="n">
-        <v>54</v>
-      </c>
-      <c r="H3" s="7" t="n">
-        <v>133</v>
+      <c r="C3" s="15" t="n">
+        <v>16</v>
+      </c>
+      <c r="D3" s="15" t="n">
+        <v>28</v>
+      </c>
+      <c r="E3" s="15" t="n">
+        <v>44</v>
+      </c>
+      <c r="F3" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="15" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
-        <is>
-          <t>Treatment</t>
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>Site</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Acidified + Ambient Temperature vs Contemporary pH + Ambient Temperature</t>
+          <t>Rainbow Reef vs Emerald Reef</t>
         </is>
       </c>
       <c r="C4" s="7" t="n">
-        <v>359</v>
+        <v>0</v>
       </c>
       <c r="D4" s="7" t="n">
-        <v>260</v>
+        <v>0</v>
       </c>
       <c r="E4" s="7" t="n">
-        <v>619</v>
+        <v>0</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>1514</v>
+        <v>0</v>
       </c>
       <c r="G4" s="7" t="n">
-        <v>2069</v>
+        <v>0</v>
       </c>
       <c r="H4" s="7" t="n">
-        <v>3583</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Contemporary pH + Bleaching vs Contemporary pH + Ambient Temperature</t>
+          <t>Star Island (Urban) vs Emerald Reef</t>
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>1715</v>
+        <v>0</v>
       </c>
       <c r="D5" s="7" t="n">
-        <v>2015</v>
+        <v>0</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>3730</v>
+        <v>0</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>1728</v>
+        <v>0</v>
       </c>
       <c r="G5" s="7" t="n">
-        <v>1997</v>
+        <v>0</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>3725</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>Acidified + Bleaching vs Contemporary pH + Ambient Temperature</t>
+          <t>MacArthur North (Urban) vs Emerald Reef</t>
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>838</v>
+        <v>34</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>1414</v>
+        <v>92</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>2252</v>
+        <v>126</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>1941</v>
+        <v>0</v>
       </c>
       <c r="G6" s="7" t="n">
-        <v>1813</v>
+        <v>0</v>
       </c>
       <c r="H6" s="7" t="n">
-        <v>3754</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>Contemporary pH + Bleaching vs Acidified + Ambient Temperature</t>
+          <t>Star Island (Urban) vs Rainbow Reef</t>
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>1416</v>
+        <v>0</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>1401</v>
+        <v>0</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>2817</v>
+        <v>0</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>6452</v>
+        <v>0</v>
       </c>
       <c r="G7" s="7" t="n">
-        <v>4149</v>
+        <v>0</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>10601</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="7" t="inlineStr">
         <is>
+          <t>MacArthur North (Urban) vs Rainbow Reef</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>123</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>164</v>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>287</v>
+      </c>
+      <c r="F8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="17" t="n"/>
+      <c r="B9" s="15" t="inlineStr">
+        <is>
+          <t>MacArthur North (Urban) vs Star Island (Urban)</t>
+        </is>
+      </c>
+      <c r="C9" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>Treatment</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Acidified + Ambient Temperature vs Contemporary pH + Ambient Temperature</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="n">
+        <v>295</v>
+      </c>
+      <c r="D10" s="7" t="n">
+        <v>102</v>
+      </c>
+      <c r="E10" s="7" t="n">
+        <v>397</v>
+      </c>
+      <c r="F10" s="7" t="n">
+        <v>1517</v>
+      </c>
+      <c r="G10" s="7" t="n">
+        <v>689</v>
+      </c>
+      <c r="H10" s="7" t="n">
+        <v>2206</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Contemporary pH + Bleaching vs Contemporary pH + Ambient Temperature</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="n">
+        <v>1728</v>
+      </c>
+      <c r="D11" s="7" t="n">
+        <v>2038</v>
+      </c>
+      <c r="E11" s="7" t="n">
+        <v>3766</v>
+      </c>
+      <c r="F11" s="7" t="n">
+        <v>1515</v>
+      </c>
+      <c r="G11" s="7" t="n">
+        <v>1871</v>
+      </c>
+      <c r="H11" s="7" t="n">
+        <v>3386</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Acidified + Bleaching vs Contemporary pH + Ambient Temperature</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="n">
+        <v>730</v>
+      </c>
+      <c r="D12" s="7" t="n">
+        <v>1184</v>
+      </c>
+      <c r="E12" s="7" t="n">
+        <v>1914</v>
+      </c>
+      <c r="F12" s="7" t="n">
+        <v>1616</v>
+      </c>
+      <c r="G12" s="7" t="n">
+        <v>1695</v>
+      </c>
+      <c r="H12" s="7" t="n">
+        <v>3311</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Contemporary pH + Bleaching vs Acidified + Ambient Temperature</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>1372</v>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>1407</v>
+      </c>
+      <c r="E13" s="7" t="n">
+        <v>2779</v>
+      </c>
+      <c r="F13" s="7" t="n">
+        <v>4643</v>
+      </c>
+      <c r="G13" s="7" t="n">
+        <v>4223</v>
+      </c>
+      <c r="H13" s="7" t="n">
+        <v>8866</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="7" t="inlineStr">
+        <is>
           <t>Acidified + Bleaching vs Contemporary pH + Bleaching</t>
         </is>
       </c>
-      <c r="C8" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="D8" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="E8" s="7" t="n">
-        <v>19</v>
-      </c>
-      <c r="F8" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="G8" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="H8" s="7" t="n">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="14" t="n"/>
-      <c r="B9" s="10" t="inlineStr">
+      <c r="C14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" s="7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="14" t="n"/>
+      <c r="B15" s="10" t="inlineStr">
         <is>
           <t>Acidified + Bleaching vs Acidified + Ambient Temperature</t>
         </is>
       </c>
-      <c r="C9" s="10" t="n">
-        <v>655</v>
-      </c>
-      <c r="D9" s="10" t="n">
-        <v>1023</v>
-      </c>
-      <c r="E9" s="10" t="n">
-        <v>1678</v>
-      </c>
-      <c r="F9" s="10" t="n">
-        <v>5853</v>
-      </c>
-      <c r="G9" s="10" t="n">
-        <v>3748</v>
-      </c>
-      <c r="H9" s="10" t="n">
-        <v>9601</v>
+      <c r="C15" s="10" t="n">
+        <v>499</v>
+      </c>
+      <c r="D15" s="10" t="n">
+        <v>903</v>
+      </c>
+      <c r="E15" s="10" t="n">
+        <v>1402</v>
+      </c>
+      <c r="F15" s="10" t="n">
+        <v>3990</v>
+      </c>
+      <c r="G15" s="10" t="n">
+        <v>3736</v>
+      </c>
+      <c r="H15" s="10" t="n">
+        <v>7726</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="C1:E1"/>
     <mergeCell ref="A4:A9"/>
     <mergeCell ref="F1:H1"/>
     <mergeCell ref="B1:B2"/>
+    <mergeCell ref="A10:A15"/>
     <mergeCell ref="A1:A2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>